<commit_message>
feat(linkml): generic workflow provenance + ai workflow provenance
</commit_message>
<xml_diff>
--- a/project/excel/fluxnova_bpm_platform.xlsx
+++ b/project/excel/fluxnova_bpm_platform.xlsx
@@ -237,7 +237,29 @@
     <sheet name="FluxnovaValue" sheetId="228" state="visible" r:id="rId228"/>
     <sheet name="BpmnModelInstance" sheetId="229" state="visible" r:id="rId229"/>
     <sheet name="BpmnModelType" sheetId="230" state="visible" r:id="rId230"/>
-    <sheet name="FluxnovaPlatformData" sheetId="231" state="visible" r:id="rId231"/>
+    <sheet name="AiAgent" sheetId="231" state="visible" r:id="rId231"/>
+    <sheet name="AiModelDescriptor" sheetId="232" state="visible" r:id="rId232"/>
+    <sheet name="AiModelInvocation" sheetId="233" state="visible" r:id="rId233"/>
+    <sheet name="PromptMessage" sheetId="234" state="visible" r:id="rId234"/>
+    <sheet name="ToolCall" sheetId="235" state="visible" r:id="rId235"/>
+    <sheet name="EvaluationResult" sheetId="236" state="visible" r:id="rId236"/>
+    <sheet name="AiDataset" sheetId="237" state="visible" r:id="rId237"/>
+    <sheet name="ModelArtifact" sheetId="238" state="visible" r:id="rId238"/>
+    <sheet name="ProvenanceBundle" sheetId="239" state="visible" r:id="rId239"/>
+    <sheet name="WorkflowDefinition" sheetId="240" state="visible" r:id="rId240"/>
+    <sheet name="StepDefinition" sheetId="241" state="visible" r:id="rId241"/>
+    <sheet name="ParameterDefinition" sheetId="242" state="visible" r:id="rId242"/>
+    <sheet name="Agent" sheetId="243" state="visible" r:id="rId243"/>
+    <sheet name="Environment" sheetId="244" state="visible" r:id="rId244"/>
+    <sheet name="RuntimeComponent" sheetId="245" state="visible" r:id="rId245"/>
+    <sheet name="WorkflowArtifact" sheetId="246" state="visible" r:id="rId246"/>
+    <sheet name="WorkflowRun" sheetId="247" state="visible" r:id="rId247"/>
+    <sheet name="StepRun" sheetId="248" state="visible" r:id="rId248"/>
+    <sheet name="ParameterValue" sheetId="249" state="visible" r:id="rId249"/>
+    <sheet name="ResourceUsage" sheetId="250" state="visible" r:id="rId250"/>
+    <sheet name="ExecutionResource" sheetId="251" state="visible" r:id="rId251"/>
+    <sheet name="ProvenanceIncident" sheetId="252" state="visible" r:id="rId252"/>
+    <sheet name="FluxnovaPlatformData" sheetId="253" state="visible" r:id="rId253"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -10485,6 +10507,1997 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:P1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>model_family</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>model_name</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>model_version</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>provider</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>endpoint</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>parameter_count</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>context_window_tokens</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>input_modalities</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>output_modalities</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>is_part_of_ai_system</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>agent_kind</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>role</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>id</t>
+        </is>
+      </c>
+      <c r="O1" t="inlineStr">
+        <is>
+          <t>name</t>
+        </is>
+      </c>
+      <c r="P1" t="inlineStr">
+        <is>
+          <t>external_ref</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <dataValidations count="3">
+    <dataValidation sqref="H2:H1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"TEXT,IMAGE,AUDIO,VIDEO,MULTIMODAL,EMBEDDING"</formula1>
+    </dataValidation>
+    <dataValidation sqref="I2:I1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"TEXT,IMAGE,AUDIO,VIDEO,MULTIMODAL,EMBEDDING"</formula1>
+    </dataValidation>
+    <dataValidation sqref="K2:K1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"PERSON,ORGANIZATION,SYSTEM,SERVICE_ACCOUNT"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet232.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:M1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>model_family</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>architecture</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>parameter_count</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>training_token_count</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>context_window_tokens</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>fine_tuning_description</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>supported_languages</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>component_kind</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>definition_version</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>endpoint</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>id</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>name</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>external_ref</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <dataValidations count="1">
+    <dataValidation sqref="H2:H1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"ENGINE,REST_API,JOB_EXECUTOR,HISTORY_EXPORTER,PLUGIN,CONNECTOR,MODELER_DEPLOYER"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet233.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:AH1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>invoked_model</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>invocation_kind</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>prompt_messages</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>tool_calls</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>response_message</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>temperature</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>top_p</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>max_tokens</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>total_input_tokens</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>total_output_tokens</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>cost_usd</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>safety_flags</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>evaluation_results</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>workflow_run</t>
+        </is>
+      </c>
+      <c r="O1" t="inlineStr">
+        <is>
+          <t>step_definition</t>
+        </is>
+      </c>
+      <c r="P1" t="inlineStr">
+        <is>
+          <t>activity_instance_id</t>
+        </is>
+      </c>
+      <c r="Q1" t="inlineStr">
+        <is>
+          <t>parent_step_run</t>
+        </is>
+      </c>
+      <c r="R1" t="inlineStr">
+        <is>
+          <t>informed_by</t>
+        </is>
+      </c>
+      <c r="S1" t="inlineStr">
+        <is>
+          <t>status</t>
+        </is>
+      </c>
+      <c r="T1" t="inlineStr">
+        <is>
+          <t>started_at</t>
+        </is>
+      </c>
+      <c r="U1" t="inlineStr">
+        <is>
+          <t>ended_at</t>
+        </is>
+      </c>
+      <c r="V1" t="inlineStr">
+        <is>
+          <t>executed_by</t>
+        </is>
+      </c>
+      <c r="W1" t="inlineStr">
+        <is>
+          <t>environment</t>
+        </is>
+      </c>
+      <c r="X1" t="inlineStr">
+        <is>
+          <t>execution_resource</t>
+        </is>
+      </c>
+      <c r="Y1" t="inlineStr">
+        <is>
+          <t>input_values</t>
+        </is>
+      </c>
+      <c r="Z1" t="inlineStr">
+        <is>
+          <t>output_values</t>
+        </is>
+      </c>
+      <c r="AA1" t="inlineStr">
+        <is>
+          <t>consumed_artifacts</t>
+        </is>
+      </c>
+      <c r="AB1" t="inlineStr">
+        <is>
+          <t>produced_artifacts</t>
+        </is>
+      </c>
+      <c r="AC1" t="inlineStr">
+        <is>
+          <t>incident_message</t>
+        </is>
+      </c>
+      <c r="AD1" t="inlineStr">
+        <is>
+          <t>retries</t>
+        </is>
+      </c>
+      <c r="AE1" t="inlineStr">
+        <is>
+          <t>sequence_no</t>
+        </is>
+      </c>
+      <c r="AF1" t="inlineStr">
+        <is>
+          <t>id</t>
+        </is>
+      </c>
+      <c r="AG1" t="inlineStr">
+        <is>
+          <t>name</t>
+        </is>
+      </c>
+      <c r="AH1" t="inlineStr">
+        <is>
+          <t>external_ref</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <dataValidations count="3">
+    <dataValidation sqref="B2:B1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"CHAT_COMPLETION,COMPLETION,EMBEDDING,TOOL_USE,AGENT_LOOP,RETRIEVAL,GUARDRAIL"</formula1>
+    </dataValidation>
+    <dataValidation sqref="L2:L1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"NONE,POLICY_VIOLATION,HALLUCINATION_SUSPECTED,JAILBREAK_ATTEMPT,PII_LEAK,PROMPT_INJECTION,TOXICITY"</formula1>
+    </dataValidation>
+    <dataValidation sqref="S2:S1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"PENDING,ACTIVE,COMPLETED,FAILED,CANCELLED,SUSPENDED"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet234.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:J1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>message_role</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>content</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>content_hash</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>sequence_no</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>redacted</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>classification</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>parent_invocation</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>id</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>name</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>external_ref</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <dataValidations count="2">
+    <dataValidation sqref="A2:A1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"SYSTEM,USER,ASSISTANT,TOOL"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F2:F1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"PUBLIC,INTERNAL,CONFIDENTIAL,RESTRICTED"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet235.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:M1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>tool_name</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>tool_call_id</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>arguments_json</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>result_json</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>result_artifact</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>called_step_run</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>started_at</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>ended_at</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>status</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>parent_invocation</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>id</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>name</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>external_ref</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <dataValidations count="1">
+    <dataValidation sqref="I2:I1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"PENDING,ACTIVE,COMPLETED,FAILED,CANCELLED,SUSPENDED"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet236.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:K1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>evaluator_name</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>evaluator_kind</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>metric_name</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>metric_value</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>metric_unit</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>passing</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>evaluated_at</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>evaluated_invocation</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>id</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>name</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>external_ref</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <dataValidations count="1">
+    <dataValidation sqref="B2:B1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"HUMAN_REVIEW,LLM_AS_JUDGE,METRIC,GUARDRAIL,STATIC_RULE"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet237.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:N1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>dataset_kind</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>record_count</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>license_uri</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>classification</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>artifact_kind</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>media_type</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>path_or_uri</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>hash</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>size_in_bytes</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>produced_by_step_run</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>consumed_by_step_runs</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>id</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>name</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>external_ref</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <dataValidations count="3">
+    <dataValidation sqref="A2:A1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"TRAINING,FINE_TUNING,EVALUATION,RAG_CORPUS,GROUND_TRUTH"</formula1>
+    </dataValidation>
+    <dataValidation sqref="D2:D1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"PUBLIC,INTERNAL,CONFIDENTIAL,RESTRICTED"</formula1>
+    </dataValidation>
+    <dataValidation sqref="E2:E1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"BPMN_XML,DMN_XML,FORM_SCHEMA,PAYLOAD,DOCUMENT,LOG,EXPORT_BUNDLE,SCREENSHOT,OTHER"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet238.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:O1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>model_card_uri</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>weights_uri</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>training_datasets</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>base_model</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>parameter_count</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>artifact_kind</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>media_type</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>path_or_uri</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>hash</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>size_in_bytes</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>produced_by_step_run</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>consumed_by_step_runs</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>id</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>name</t>
+        </is>
+      </c>
+      <c r="O1" t="inlineStr">
+        <is>
+          <t>external_ref</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <dataValidations count="1">
+    <dataValidation sqref="F2:F1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"BPMN_XML,DMN_XML,FORM_SCHEMA,PAYLOAD,DOCUMENT,LOG,EXPORT_BUNDLE,SCREENSHOT,OTHER"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet239.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:M1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>id</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>name</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>generated_at</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>source_system</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>schema_version</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>workflow_definitions</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>workflow_runs</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>agents</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>environments</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>runtime_components</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>workflow_artifacts</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>parameter_values</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>resources</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet24.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>id</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>resource_type</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>name</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>owner</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>query</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>properties</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet240.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:K1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>definition_version</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>definition_key</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>deployment_id</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>source_model_ref</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>runtime_component</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>steps</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>authors</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>tags</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>id</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>name</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>external_ref</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet241.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:M1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>workflow_definition</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>bpmn_type</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>implementation_kind</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>implementation_ref</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>called_element</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>decision_ref</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>form_ref</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>input_parameters</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>output_parameters</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>bpmn_extension_names</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>id</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>name</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>external_ref</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <dataValidations count="1">
+    <dataValidation sqref="C2:C1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"USER_TASK,JAVA_DELEGATE,EXPRESSION,SCRIPT,CONNECTOR,CALL_ACTIVITY,BUSINESS_RULE,EXTERNAL_SERVICE,EVENT,GATEWAY,SUBPROCESS"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet242.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:J1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>parameter_scope</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>parameter_direction</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>declared_type</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>is_required</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>default_value</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>secret</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>allowed_values</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>id</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>name</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>external_ref</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <dataValidations count="2">
+    <dataValidation sqref="A2:A1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"WORKFLOW,STEP,TASK,DECISION,FORM"</formula1>
+    </dataValidation>
+    <dataValidation sqref="B2:B1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"IN,OUT,INOUT,LOCAL"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet243.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>agent_kind</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>role</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>id</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>name</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>external_ref</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <dataValidations count="1">
+    <dataValidation sqref="A2:A1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"PERSON,ORGANIZATION,SYSTEM,SERVICE_ACCOUNT"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet244.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>runtime_name</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>runtime_version</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>host</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>region</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>deployment_ref</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>configuration_ref</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>id</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>name</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>external_ref</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet245.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>component_kind</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>definition_version</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>endpoint</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>id</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>name</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>external_ref</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <dataValidations count="1">
+    <dataValidation sqref="A2:A1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"ENGINE,REST_API,JOB_EXECUTOR,HISTORY_EXPORTER,PLUGIN,CONNECTOR,MODELER_DEPLOYER"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet246.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:J1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>artifact_kind</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>media_type</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>path_or_uri</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>hash</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>size_in_bytes</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>produced_by_step_run</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>consumed_by_step_runs</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>id</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>name</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>external_ref</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <dataValidations count="1">
+    <dataValidation sqref="A2:A1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"BPMN_XML,DMN_XML,FORM_SCHEMA,PAYLOAD,DOCUMENT,LOG,EXPORT_BUNDLE,SCREENSHOT,OTHER"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet247.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:R1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>workflow_definition</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>business_key</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>parent_workflow_run</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>status</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>started_at</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>ended_at</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>started_by</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>environment</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>runtime_component</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>input_values</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>output_values</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>step_runs</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>incidents</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>resource_usage</t>
+        </is>
+      </c>
+      <c r="O1" t="inlineStr">
+        <is>
+          <t>tags</t>
+        </is>
+      </c>
+      <c r="P1" t="inlineStr">
+        <is>
+          <t>id</t>
+        </is>
+      </c>
+      <c r="Q1" t="inlineStr">
+        <is>
+          <t>name</t>
+        </is>
+      </c>
+      <c r="R1" t="inlineStr">
+        <is>
+          <t>external_ref</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <dataValidations count="1">
+    <dataValidation sqref="D2:D1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"PENDING,ACTIVE,COMPLETED,FAILED,CANCELLED,SUSPENDED"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet248.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:U1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>workflow_run</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>step_definition</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>activity_instance_id</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>parent_step_run</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>informed_by</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>status</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>started_at</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>ended_at</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>executed_by</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>environment</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>execution_resource</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>input_values</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>output_values</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>consumed_artifacts</t>
+        </is>
+      </c>
+      <c r="O1" t="inlineStr">
+        <is>
+          <t>produced_artifacts</t>
+        </is>
+      </c>
+      <c r="P1" t="inlineStr">
+        <is>
+          <t>incident_message</t>
+        </is>
+      </c>
+      <c r="Q1" t="inlineStr">
+        <is>
+          <t>retries</t>
+        </is>
+      </c>
+      <c r="R1" t="inlineStr">
+        <is>
+          <t>sequence_no</t>
+        </is>
+      </c>
+      <c r="S1" t="inlineStr">
+        <is>
+          <t>id</t>
+        </is>
+      </c>
+      <c r="T1" t="inlineStr">
+        <is>
+          <t>name</t>
+        </is>
+      </c>
+      <c r="U1" t="inlineStr">
+        <is>
+          <t>external_ref</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <dataValidations count="1">
+    <dataValidation sqref="F2:F1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"PENDING,ACTIVE,COMPLETED,FAILED,CANCELLED,SUSPENDED"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet249.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:N1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>parameter_definition</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>observed_type</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>parameter_direction</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>serialized_value</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>value_hash</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>observed_at</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>produced_by_step_run</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>consumed_by_step_runs</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>derived_from</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>redacted</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>classification</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>id</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>name</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>external_ref</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <dataValidations count="2">
+    <dataValidation sqref="C2:C1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"IN,OUT,INOUT,LOCAL"</formula1>
+    </dataValidation>
+    <dataValidation sqref="K2:K1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"PUBLIC,INTERNAL,CONFIDENTIAL,RESTRICTED"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet25.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:J1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>id</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>key</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>name</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>version</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>category</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>deployment_id</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>resource_name</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>diagram_resource_name</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>tenant_id</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>history_time_to_live</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet250.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>metric_name</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>metric_value</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>metric_unit</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>measured_for_workflow_run</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>measured_for_step_run</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>execution_resource</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>id</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>name</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>external_ref</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet251.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>resource_kind</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>host</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>endpoint</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>labels</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>id</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>name</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>external_ref</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <dataValidations count="1">
+    <dataValidation sqref="A2:A1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"HOST,CONTAINER,POD,NODE,DATABASE,QUEUE,CLUSTER,THREAD_POOL,EXTERNAL_API"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet252.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>incident_status</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>message</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>observed_at</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>related_step_run</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>related_workflow_run</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>id</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>name</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>external_ref</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <dataValidations count="1">
+    <dataValidation sqref="A2:A1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"OPEN,INVESTIGATING,RESOLVED,IGNORED"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet253.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:H1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
@@ -10527,118 +12540,6 @@
       <c r="H1" t="inlineStr">
         <is>
           <t>batches</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet24.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:F1"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>id</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>resource_type</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>name</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>owner</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>query</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>properties</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet25.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:J1"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>id</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>key</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>name</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>version</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>category</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>deployment_id</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>resource_name</t>
-        </is>
-      </c>
-      <c r="H1" t="inlineStr">
-        <is>
-          <t>diagram_resource_name</t>
-        </is>
-      </c>
-      <c r="I1" t="inlineStr">
-        <is>
-          <t>tenant_id</t>
-        </is>
-      </c>
-      <c r="J1" t="inlineStr">
-        <is>
-          <t>history_time_to_live</t>
         </is>
       </c>
     </row>

</xml_diff>